<commit_message>
Panel namunasi: ariza holati maydonlari
</commit_message>
<xml_diff>
--- a/panel/arizalar.xlsx
+++ b/panel/arizalar.xlsx
@@ -490,7 +490,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-10-15 05:34:18</t>
+          <t>2026-10-15 05:35:26</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -536,7 +536,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-10-14 22:34:18</t>
+          <t>2026-10-14 22:35:26</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -578,7 +578,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2026-10-14 15:34:18</t>
+          <t>2026-10-14 15:35:26</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -624,7 +624,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-10-14 08:34:18</t>
+          <t>2026-10-14 08:35:26</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2026-10-14 01:34:18</t>
+          <t>2026-10-14 01:35:26</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -720,7 +720,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-10-13 18:34:18</t>
+          <t>2026-10-13 18:35:26</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">

</xml_diff>

<commit_message>
Panel namunasi: tanlash ro'yxatlari panel uslubida
</commit_message>
<xml_diff>
--- a/panel/arizalar.xlsx
+++ b/panel/arizalar.xlsx
@@ -914,7 +914,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>«Oltinko‘l tuman charm-poyabzal kichik sanoat zonasini boshqarish direksiyasi» MChJ · 15.10.2026 13:00 holatiga · jami 6 ta</t>
+          <t>«Oltinko‘l tuman charm-poyabzal kichik sanoat zonasini boshqarish direksiyasi» MChJ · 15.10.2026 14:37 holatiga · jami 6 ta</t>
         </is>
       </c>
     </row>
@@ -980,7 +980,7 @@
         <v>6</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>46310.25</v>
+        <v>46310.31736111111</v>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
@@ -1015,7 +1015,7 @@
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>2026-10-15 13:00 · Direksiya (namuna): Qo‘ng‘iroq qildim, ma’lumot berdim</t>
+          <t>2026-10-15 14:37 · Direksiya (namuna): Qo‘ng‘iroq qildim, ma’lumot berdim</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1029,7 +1029,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>46309.95833333334</v>
+        <v>46310.02569444444</v>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
@@ -1070,7 +1070,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="5" t="n">
-        <v>46309.66666666666</v>
+        <v>46309.73402777778</v>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
@@ -1115,7 +1115,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="5" t="n">
-        <v>46309.375</v>
+        <v>46309.44236111111</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>2026-10-15 13:00 · Direksiya (namuna): Qo‘ng‘iroq qildim, ma’lumot berdim</t>
+          <t>2026-10-15 14:37 · Direksiya (namuna): Qo‘ng‘iroq qildim, ma’lumot berdim</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
@@ -1164,7 +1164,7 @@
         <v>2</v>
       </c>
       <c r="B9" s="5" t="n">
-        <v>46309.08333333334</v>
+        <v>46309.15069444444</v>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
@@ -1203,7 +1203,7 @@
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>2026-10-15 13:00 · Direksiya (namuna): Qo‘ng‘iroq qildim, ma’lumot berdim</t>
+          <t>2026-10-15 14:37 · Direksiya (namuna): Qo‘ng‘iroq qildim, ma’lumot berdim</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -1217,7 +1217,7 @@
         <v>1</v>
       </c>
       <c r="B10" s="5" t="n">
-        <v>46308.79166666666</v>
+        <v>46308.85902777778</v>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>2026-10-15 13:00 · Direksiya (namuna): Qo‘ng‘iroq qildim, ma’lumot berdim</t>
+          <t>2026-10-15 14:37 · Direksiya (namuna): Qo‘ng‘iroq qildim, ma’lumot berdim</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>«Oltinko‘l tuman charm-poyabzal kichik sanoat zonasini boshqarish direksiyasi» MChJ · 15.10.2026 13:00 holatiga</t>
+          <t>«Oltinko‘l tuman charm-poyabzal kichik sanoat zonasini boshqarish direksiyasi» MChJ · 15.10.2026 14:37 holatiga</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tanlash ro'yxati: variant bosilganda yopiladi
</commit_message>
<xml_diff>
--- a/panel/arizalar.xlsx
+++ b/panel/arizalar.xlsx
@@ -914,7 +914,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>«Oltinko‘l tuman charm-poyabzal kichik sanoat zonasini boshqarish direksiyasi» MChJ · 15.10.2026 14:37 holatiga · jami 6 ta</t>
+          <t>«Oltinko‘l tuman charm-poyabzal kichik sanoat zonasini boshqarish direksiyasi» MChJ · 15.10.2026 14:39 holatiga · jami 6 ta</t>
         </is>
       </c>
     </row>
@@ -980,7 +980,7 @@
         <v>6</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>46310.31736111111</v>
+        <v>46310.31875</v>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
@@ -1015,7 +1015,7 @@
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>2026-10-15 14:37 · Direksiya (namuna): Qo‘ng‘iroq qildim, ma’lumot berdim</t>
+          <t>2026-10-15 14:39 · Direksiya (namuna): Qo‘ng‘iroq qildim, ma’lumot berdim</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1029,7 +1029,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>46310.02569444444</v>
+        <v>46310.02708333333</v>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
@@ -1070,7 +1070,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="5" t="n">
-        <v>46309.73402777778</v>
+        <v>46309.73541666667</v>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
@@ -1115,7 +1115,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="5" t="n">
-        <v>46309.44236111111</v>
+        <v>46309.44375</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>2026-10-15 14:37 · Direksiya (namuna): Qo‘ng‘iroq qildim, ma’lumot berdim</t>
+          <t>2026-10-15 14:39 · Direksiya (namuna): Qo‘ng‘iroq qildim, ma’lumot berdim</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
@@ -1164,7 +1164,7 @@
         <v>2</v>
       </c>
       <c r="B9" s="5" t="n">
-        <v>46309.15069444444</v>
+        <v>46309.15208333333</v>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
@@ -1203,7 +1203,7 @@
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>2026-10-15 14:37 · Direksiya (namuna): Qo‘ng‘iroq qildim, ma’lumot berdim</t>
+          <t>2026-10-15 14:39 · Direksiya (namuna): Qo‘ng‘iroq qildim, ma’lumot berdim</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -1217,7 +1217,7 @@
         <v>1</v>
       </c>
       <c r="B10" s="5" t="n">
-        <v>46308.85902777778</v>
+        <v>46308.86041666667</v>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>2026-10-15 14:37 · Direksiya (namuna): Qo‘ng‘iroq qildim, ma’lumot berdim</t>
+          <t>2026-10-15 14:39 · Direksiya (namuna): Qo‘ng‘iroq qildim, ma’lumot berdim</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>«Oltinko‘l tuman charm-poyabzal kichik sanoat zonasini boshqarish direksiyasi» MChJ · 15.10.2026 14:37 holatiga</t>
+          <t>«Oltinko‘l tuman charm-poyabzal kichik sanoat zonasini boshqarish direksiyasi» MChJ · 15.10.2026 14:39 holatiga</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Panel namunasi: qidiruv lotin/kirillda
</commit_message>
<xml_diff>
--- a/panel/arizalar.xlsx
+++ b/panel/arizalar.xlsx
@@ -914,7 +914,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>«Oltinko‘l tuman charm-poyabzal kichik sanoat zonasini boshqarish direksiyasi» MChJ · 15.10.2026 14:39 holatiga · jami 6 ta</t>
+          <t>«Oltinko‘l tuman charm-poyabzal kichik sanoat zonasini boshqarish direksiyasi» MChJ · 15.10.2026 16:26 holatiga · jami 6 ta</t>
         </is>
       </c>
     </row>
@@ -980,7 +980,7 @@
         <v>6</v>
       </c>
       <c r="B5" s="5" t="n">
-        <v>46310.31875</v>
+        <v>46310.39305555556</v>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
@@ -1015,7 +1015,7 @@
       </c>
       <c r="J5" s="7" t="inlineStr">
         <is>
-          <t>2026-10-15 14:39 · Direksiya (namuna): Qo‘ng‘iroq qildim, ma’lumot berdim</t>
+          <t>2026-10-15 16:26 · Direksiya (namuna): Qo‘ng‘iroq qildim, ma’lumot berdim</t>
         </is>
       </c>
       <c r="K5" s="4" t="inlineStr">
@@ -1029,7 +1029,7 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="n">
-        <v>46310.02708333333</v>
+        <v>46310.10138888889</v>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
@@ -1070,7 +1070,7 @@
         <v>4</v>
       </c>
       <c r="B7" s="5" t="n">
-        <v>46309.73541666667</v>
+        <v>46309.80972222222</v>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
@@ -1115,7 +1115,7 @@
         <v>3</v>
       </c>
       <c r="B8" s="5" t="n">
-        <v>46309.44375</v>
+        <v>46309.51805555556</v>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
@@ -1150,7 +1150,7 @@
       </c>
       <c r="J8" s="7" t="inlineStr">
         <is>
-          <t>2026-10-15 14:39 · Direksiya (namuna): Qo‘ng‘iroq qildim, ma’lumot berdim</t>
+          <t>2026-10-15 16:26 · Direksiya (namuna): Qo‘ng‘iroq qildim, ma’lumot berdim</t>
         </is>
       </c>
       <c r="K8" s="4" t="inlineStr">
@@ -1164,7 +1164,7 @@
         <v>2</v>
       </c>
       <c r="B9" s="5" t="n">
-        <v>46309.15208333333</v>
+        <v>46309.22638888889</v>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
@@ -1203,7 +1203,7 @@
       </c>
       <c r="J9" s="7" t="inlineStr">
         <is>
-          <t>2026-10-15 14:39 · Direksiya (namuna): Qo‘ng‘iroq qildim, ma’lumot berdim</t>
+          <t>2026-10-15 16:26 · Direksiya (namuna): Qo‘ng‘iroq qildim, ma’lumot berdim</t>
         </is>
       </c>
       <c r="K9" s="4" t="inlineStr">
@@ -1217,7 +1217,7 @@
         <v>1</v>
       </c>
       <c r="B10" s="5" t="n">
-        <v>46308.86041666667</v>
+        <v>46308.93472222222</v>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
@@ -1256,7 +1256,7 @@
       </c>
       <c r="J10" s="7" t="inlineStr">
         <is>
-          <t>2026-10-15 14:39 · Direksiya (namuna): Qo‘ng‘iroq qildim, ma’lumot berdim</t>
+          <t>2026-10-15 16:26 · Direksiya (namuna): Qo‘ng‘iroq qildim, ma’lumot berdim</t>
         </is>
       </c>
       <c r="K10" s="4" t="inlineStr">
@@ -1307,7 +1307,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>«Oltinko‘l tuman charm-poyabzal kichik sanoat zonasini boshqarish direksiyasi» MChJ · 15.10.2026 14:39 holatiga</t>
+          <t>«Oltinko‘l tuman charm-poyabzal kichik sanoat zonasini boshqarish direksiyasi» MChJ · 15.10.2026 16:26 holatiga</t>
         </is>
       </c>
     </row>

</xml_diff>